<commit_message>
자동 갱신 2026-10-18 17:55
</commit_message>
<xml_diff>
--- a/files/thebookman-booklist.xlsx
+++ b/files/thebookman-booklist.xlsx
@@ -535,54 +535,54 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>여름</t>
+          <t>품격 있는 대화를 위한 지식 브리핑 (10만 부 기념 특별 한정판)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>이디스 워튼 (지은이), 민지현 (옮긴이)</t>
+          <t>김진 (지은이)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>머묾</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>19000</v>
+        <v>25000</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>9791124038802</t>
+          <t>9791124038413</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401985055</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=404263026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>위대한 개츠비</t>
+          <t>여름</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>프랜시스 스콧 피츠제럴드 (지은이), 이미정 (옮긴이)</t>
+          <t>이디스 워튼 (지은이), 민지현 (옮긴이)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -605,25 +605,25 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>9791124038659</t>
+          <t>9791124038802</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401984756</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401985055</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>파리는 언제나 축제</t>
+          <t>위대한 개츠비</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>어니스트 헤밍웨이 (지은이), 권진아 (옮긴이)</t>
+          <t>프랜시스 스콧 피츠제럴드 (지은이), 이미정 (옮긴이)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -646,39 +646,35 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>9791124038666</t>
+          <t>9791124038659</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401985497</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401984756</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>단단히, 휩쓸리지 않고 살아간다는 것</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>흔들리는 시간을 지혜롭게 건너는 마음의 철학</t>
-        </is>
-      </c>
+          <t>파리는 언제나 축제</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>나디 미리안 (지은이), 김지유 (옮긴이)</t>
+          <t>어니스트 헤밍웨이 (지은이), 권진아 (옮긴이)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>머묾</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -687,88 +683,88 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>22000</v>
+        <v>19000</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>9791124038888</t>
+          <t>9791124038666</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=403488397</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401985497</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>머니 트렌드 2027</t>
+          <t>단단히, 휩쓸리지 않고 살아간다는 것</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>격변의 위기를 기회로 바꾸는 55가지 돈의 흐름</t>
+          <t>흔들리는 시간을 지혜롭게 건너는 마음의 철학</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>정태익, 김도윤, 김광석, 김용섭, 김학렬, 박세익, 박정호, 이효석 (지은이)</t>
+          <t>나디 미리안 (지은이), 김지유 (옮긴이)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>27500</v>
+        <v>22000</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>9791124038826</t>
+          <t>9791124038888</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401122536</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=403488397</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>처음 만나는 철학의 세계</t>
+          <t>머니 트렌드 2027</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>삶에 철학이 들어오는 순간</t>
+          <t>격변의 위기를 기회로 바꾸는 55가지 돈의 흐름</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>성창원 (지은이)</t>
+          <t>정태익, 김도윤, 김광석, 김용섭, 김학렬, 박세익, 박정호, 이효석 (지은이)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -777,33 +773,33 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>22000</v>
+        <v>27500</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>9791124038833</t>
+          <t>9791124038826</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=402017704</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=401122536</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>똑똑한 사람은 어떻게 말하는가</t>
+          <t>처음 만나는 철학의 세계</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>길게 말하지 않아도 신뢰받는 사람들의 말하기 전략</t>
+          <t>삶에 철학이 들어오는 순간</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>이시한 (지은이)</t>
+          <t>성창원 (지은이)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -813,12 +809,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -826,171 +822,175 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>9791124038642</t>
+          <t>9791124038833</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=400007561</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=402017704</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>기억의 무늬</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>똑똑한 사람은 어떻게 말하는가</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>길게 말하지 않아도 신뢰받는 사람들의 말하기 전략</t>
+        </is>
+      </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>백희성 (지은이)</t>
+          <t>이시한 (지은이)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>19800</v>
+        <v>22000</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>9791124038604</t>
+          <t>9791124038642</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=398993923</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=400007561</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>나는 도대체 왜 눈치를 볼까</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>타인의 기대에서 벗어나 원하는 삶을 사는 법</t>
-        </is>
-      </c>
+          <t>기억의 무늬</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>케리 올리치, 켈리 권터 (지은이), 김잔디 (옮긴이)</t>
+          <t>백희성 (지은이)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>21000</v>
+        <v>19800</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>9791124038536</t>
+          <t>9791124038604</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=397995935</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=398993923</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>만일 나에게 단 한 번의 아침이 남아 있다면 (굿모닝 에디션)</t>
+          <t>나는 도대체 왜 눈치를 볼까</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>오늘이 끝나기 전 반드시 깨달아야 할 것들</t>
+          <t>타인의 기대에서 벗어나 원하는 삶을 사는 법</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>존 릴런드 (지은이), 최인하 (옮긴이)</t>
+          <t>케리 올리치, 켈리 권터 (지은이), 김잔디 (옮긴이)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>19800</v>
+        <v>21000</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>9791193937112</t>
+          <t>9791124038536</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=398820063</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=397995935</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>너의 행복은 나의 기쁨이야</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t>만일 나에게 단 한 번의 아침이 남아 있다면 (굿모닝 에디션)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>오늘이 끝나기 전 반드시 깨달아야 할 것들</t>
+        </is>
+      </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>정한경 (지은이)</t>
+          <t>존 릴런드 (지은이), 최인하 (옮긴이)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -998,80 +998,76 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>9791124038574</t>
+          <t>9791193937112</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396794390</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=398820063</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>여름 (썸머 에디션)</t>
+          <t>너의 행복은 나의 기쁨이야</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>이디스 워튼 (지은이), 민지현 (옮긴이)</t>
+          <t>정한경 (지은이)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>머묾</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>19000</v>
+        <v>19800</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>9791124038581</t>
+          <t>9791124038574</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396568091</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396794390</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>끌리는 사람의 비밀</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>마음을 움직이는 품위 있는 말과 태도</t>
-        </is>
-      </c>
+          <t>여름 (썸머 에디션)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>조수빈 (지은이)</t>
+          <t>이디스 워튼 (지은이), 민지현 (옮긴이)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>머묾</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1080,38 +1076,38 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>22000</v>
+        <v>19000</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>9791124038567</t>
+          <t>9791124038581</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396156367</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396568091</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>최소한의 습관</t>
+          <t>끌리는 사람의 비밀</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>작은 시작으로 압도적 변화를 만드는 행동 공식</t>
+          <t>마음을 움직이는 품위 있는 말과 태도</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>로버트 마우어 (지은이), 장원철 (옮긴이)</t>
+          <t>조수빈 (지은이)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1121,74 +1117,78 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>19800</v>
+        <v>22000</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>9791124038512</t>
+          <t>9791124038567</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=394919714</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396156367</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>이방인</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t>최소한의 습관</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>작은 시작으로 압도적 변화를 만드는 행동 공식</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>알베르 카뮈 (지은이), 한수민 (옮긴이)</t>
+          <t>로버트 마우어 (지은이), 장원철 (옮긴이)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>머묾</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>9791124038390</t>
+          <t>9791124038512</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396164215</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=394919714</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>프랑켄슈타인</t>
+          <t>이방인</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>메리 셸리 (지은이), 이미애 (옮긴이)</t>
+          <t>알베르 카뮈 (지은이), 한수민 (옮긴이)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1207,29 +1207,29 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>21000</v>
+        <v>18000</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>9791124038383</t>
+          <t>9791124038390</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396166191</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396164215</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>올랜도</t>
+          <t>프랑켄슈타인</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>버지니아 울프 (지은이), 정해영 (옮긴이)</t>
+          <t>메리 셸리 (지은이), 이미애 (옮긴이)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1248,34 +1248,34 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>9791124038406</t>
+          <t>9791124038383</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396167382</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396166191</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>리치먼드힐의 이층 버스</t>
+          <t>올랜도</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>이경진 (지은이)</t>
+          <t>버지니아 울프 (지은이), 정해영 (옮긴이)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>머묾</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1289,188 +1289,188 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>19000</v>
+        <v>20000</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>9791124038499</t>
+          <t>9791124038406</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=394084608</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=396167382</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>밤의 설계자</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>잠들기 전 15분, 미래를 바꾸는 밤 생각 습관</t>
-        </is>
-      </c>
+          <t>리치먼드힐의 이층 버스</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
-          <t>폴커 부슈 (지은이), 이상희 (옮긴이)</t>
+          <t>이경진 (지은이)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>22000</v>
+        <v>19000</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>9791124038468</t>
+          <t>9791124038499</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=393318252</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=394084608</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>웨딩 피플</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
+          <t>밤의 설계자</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>잠들기 전 15분, 미래를 바꾸는 밤 생각 습관</t>
+        </is>
+      </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>앨리슨 에스파흐 (지은이), 김보람 (옮긴이)</t>
+          <t>폴커 부슈 (지은이), 이상희 (옮긴이)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>9791124038437</t>
+          <t>9791124038468</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=392621945</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=393318252</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>아우슈비츠의 무용수</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>인생은 언제나 다시 선택할 수 있다</t>
-        </is>
-      </c>
+          <t>웨딩 피플</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>에디트 에바 에거 (지은이), 안진희 (옮긴이)</t>
+          <t>앨리슨 에스파흐 (지은이), 김보람 (옮긴이)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>24000</v>
+        <v>21000</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>9791124038352</t>
+          <t>9791124038437</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=391538652</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=392621945</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>품격 있는 대화를 위한 지식 브리핑 (10만 부 기념 특별 한정판)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>아우슈비츠의 무용수</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>인생은 언제나 다시 선택할 수 있다</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>김진 (지은이)</t>
+          <t>에디트 에바 에거 (지은이), 안진희 (옮긴이)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>25000</v>
+        <v>24000</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>9791124038413</t>
+          <t>9791124038352</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=404263026</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=391538652</t>
         </is>
       </c>
     </row>
@@ -5723,37 +5723,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Money Trend 2027</t>
+          <t>A Briefing on Knowledge for Conversations Worth Having (Special Limited Edition)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>55 currents of money that turn upheaval into opportunity.</t>
+          <t>The knowledge behind thoughtful, well-informed conversation.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>머니 트렌드 2027</t>
+          <t>품격 있는 대화를 위한 지식 브리핑 (10만 부 기념 특별 한정판)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>정태익, 김도윤, 김광석, 김용섭, 김학렬, 박세익, 박정호, 이효석</t>
+          <t>김진</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Humanities</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>9791124038826</t>
+          <t>9791124038413</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -5765,27 +5765,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Meeting Philosophy for the First Time</t>
+          <t>Money Trend 2027</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The moment philosophy walks into your life.</t>
+          <t>55 currents of money that turn upheaval into opportunity.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>처음 만나는 철학의 세계</t>
+          <t>머니 트렌드 2027</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>성창원</t>
+          <t>정태익, 김도윤, 김광석, 김용섭, 김학렬, 박세익, 박정호, 이효석</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Humanities</t>
+          <t>Business</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>9791124038833</t>
+          <t>9791124038826</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -5807,37 +5807,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>How Smart People Talk</t>
+          <t>Meeting Philosophy for the First Time</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Speaking strategies of people who earn trust without talking long.</t>
+          <t>The moment philosophy walks into your life.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>똑똑한 사람은 어떻게 말하는가</t>
+          <t>처음 만나는 철학의 세계</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>이시한</t>
+          <t>성창원</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Self-Help</t>
+          <t>Humanities</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>9791124038642</t>
+          <t>9791124038833</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5849,37 +5849,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The Texture of Memory</t>
+          <t>How Smart People Talk</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unable to recognize faces, she reads people through cloth and gait.</t>
+          <t>Speaking strategies of people who earn trust without talking long.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>기억의 무늬</t>
+          <t>똑똑한 사람은 어떻게 말하는가</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>백희성</t>
+          <t>이시한</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>Self-Help</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>9791124038604</t>
+          <t>9791124038642</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5891,37 +5891,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Your Happiness Is My Joy</t>
+          <t>The Texture of Memory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>To love someone is to find your joy in theirs.</t>
+          <t>Unable to recognize faces, she reads people through cloth and gait.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>너의 행복은 나의 기쁨이야</t>
+          <t>기억의 무늬</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>정한경</t>
+          <t>백희성</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Essay</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>9791124038574</t>
+          <t>9791124038604</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -5933,37 +5933,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>The Secret of Magnetic People</t>
+          <t>Your Happiness Is My Joy</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Graceful words and bearing that move hearts.</t>
+          <t>To love someone is to find your joy in theirs.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>끌리는 사람의 비밀</t>
+          <t>너의 행복은 나의 기쁨이야</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>조수빈</t>
+          <t>정한경</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Self-Help</t>
+          <t>Essay</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>9791124038567</t>
+          <t>9791124038574</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -5975,37 +5975,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The Double-Decker Bus of Richmond Hill</t>
+          <t>The Secret of Magnetic People</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>If you could change the past, would you choose differently?</t>
+          <t>Graceful words and bearing that move hearts.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>리치먼드힐의 이층 버스</t>
+          <t>끌리는 사람의 비밀</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>이경진</t>
+          <t>조수빈</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fiction</t>
+          <t>Self-Help</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>9791124038499</t>
+          <t>9791124038567</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -6017,37 +6017,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A Briefing on Knowledge for Conversations Worth Having (Special Limited Edition)</t>
+          <t>The Double-Decker Bus of Richmond Hill</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The knowledge behind thoughtful, well-informed conversation.</t>
+          <t>If you could change the past, would you choose differently?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>품격 있는 대화를 위한 지식 브리핑 (10만 부 기념 특별 한정판)</t>
+          <t>리치먼드힐의 이층 버스</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>김진</t>
+          <t>이경진</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Humanities</t>
+          <t>Fiction</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9791124038413</t>
+          <t>9791124038499</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">

</xml_diff>

<commit_message>
자동 갱신 2026-10-19 09:55
</commit_message>
<xml_diff>
--- a/files/thebookman-booklist.xlsx
+++ b/files/thebookman-booklist.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3676,72 +3676,72 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>새들이 남쪽으로 가는 날</t>
+          <t>왜 그들만 부자가 되는가</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2024 스웨덴 올해의 도서상 수상작</t>
+          <t>부의 격차를 좁히는 진짜 돈의 모습</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>리사 리드센 (지은이), 손화수 (옮긴이)</t>
+          <t>필립 바구스, 안드레아스 마르크바르트 (지은이), 배진아 (옮긴이)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2024-12-18</t>
+          <t>2025-01-08</t>
         </is>
       </c>
       <c r="G76" t="n">
-        <v>19500</v>
+        <v>22000</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>9791193937372</t>
+          <t>9791193937396</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=352764746</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=354574933</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>삶의 태도</t>
+          <t>새들이 남쪽으로 가는 날</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>흔들림 없이 나아가는</t>
+          <t>2024 스웨덴 올해의 도서상 수상작</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>반건호 (지은이)</t>
+          <t>리사 리드센 (지은이), 손화수 (옮긴이)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3750,213 +3750,213 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>22000</v>
+        <v>19500</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>9791193937402</t>
+          <t>9791193937372</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=353472576</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=352764746</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>인생을 자유롭게 하는 것들</t>
+          <t>삶의 태도</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>가슴 뛰는 삶을 향해 가는 최우선의 행복</t>
+          <t>흔들림 없이 나아가는</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>나용민, 유숙현 (지은이)</t>
+          <t>반건호 (지은이)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2024-12-13</t>
+          <t>2024-12-18</t>
         </is>
       </c>
       <c r="G78" t="n">
-        <v>18000</v>
+        <v>22000</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>9791193937389</t>
+          <t>9791193937402</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=353117247</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=353472576</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>쉼과 나아감에 대하여</t>
+          <t>인생을 자유롭게 하는 것들</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>인생의 오아시스를 만나는 예일대 명강의</t>
+          <t>가슴 뛰는 삶을 향해 가는 최우선의 행복</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>마릴린 폴 (지은이), 김태훈 (옮긴이)</t>
+          <t>나용민, 유숙현 (지은이)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2024-11-27</t>
+          <t>2024-12-13</t>
         </is>
       </c>
       <c r="G79" t="n">
-        <v>19800</v>
+        <v>18000</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>9791193937341</t>
+          <t>9791193937389</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=351959853</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=353117247</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>영국 아빠 피터의 하루 3분 영어 대화 (스프링)</t>
+          <t>쉼과 나아감에 대하여</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>스스로 말하고 표현하는 영어 회화 일력</t>
+          <t>인생의 오아시스를 만나는 예일대 명강의</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>피터 빈트 (지은이)</t>
+          <t>마릴린 폴 (지은이), 김태훈 (옮긴이)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>북크레용</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>자녀교육</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2024-10-23</t>
+          <t>2024-11-27</t>
         </is>
       </c>
       <c r="G80" t="n">
-        <v>25000</v>
+        <v>19800</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>9791193937280</t>
+          <t>9791193937341</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=350405920</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=351959853</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>질투라는 감옥</t>
+          <t>영국 아빠 피터의 하루 3분 영어 대화 (스프링)</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>우리는 왜 타인에게 휘둘리는가</t>
+          <t>스스로 말하고 표현하는 영어 회화 일력</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>야마모토 케이 (지은이), 최주연 (옮긴이)</t>
+          <t>피터 빈트 (지은이)</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북크레용</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>자녀교육</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2024-10-16</t>
+          <t>2024-10-23</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>19800</v>
+        <v>25000</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>9791193937259</t>
+          <t>9791193937280</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=348985847</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=350405920</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>머니 트렌드 2025</t>
+          <t>질투라는 감옥</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>새로운 부의 기회를 선점할 55가지 성공 시나리오</t>
+          <t>우리는 왜 타인에게 휘둘리는가</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>정태익, 김도윤, 김광석, 김용섭, 김현준, 정수종, 채상욱, 최재붕 (지은이)</t>
+          <t>야마모토 케이 (지은이), 최주연 (옮긴이)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3966,143 +3966,147 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2024-10-02</t>
+          <t>2024-10-16</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>25000</v>
+        <v>19800</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>9791193937211</t>
+          <t>9791193937259</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=345965820</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=348985847</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>마음이 부자인 아이는 어떻게 성장하는가</t>
+          <t>머니 트렌드 2025</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>행복할 줄 아는 아이로 키우는 정서 육아법</t>
+          <t>새로운 부의 기회를 선점할 55가지 성공 시나리오</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>박소영 (지은이)</t>
+          <t>정태익, 김도윤, 김광석, 김용섭, 김현준, 정수종, 채상욱, 최재붕 (지은이)</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>북크레용</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>자녀교육</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2024-09-25</t>
+          <t>2024-10-02</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>19800</v>
+        <v>25000</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>9791193937228</t>
+          <t>9791193937211</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=346892914</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=345965820</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>엄마에게 안부를 묻는 밤</t>
+          <t>마음이 부자인 아이는 어떻게 성장하는가</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>언제나 내 편인 이 세상 단 한 사람</t>
+          <t>행복할 줄 아는 아이로 키우는 정서 육아법</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>박애희 (지은이)</t>
+          <t>박소영 (지은이)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>북파머스</t>
+          <t>북크레용</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>자녀교육</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2024-09-19</t>
+          <t>2024-09-25</t>
         </is>
       </c>
       <c r="G84" t="n">
-        <v>18800</v>
+        <v>19800</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>9791193937242</t>
+          <t>9791193937228</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=346467345</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=346892914</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>빛이 이끄는 곳으로</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr"/>
+          <t>엄마에게 안부를 묻는 밤</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>언제나 내 편인 이 세상 단 한 사람</t>
+        </is>
+      </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>백희성 (지은이)</t>
+          <t>박애희 (지은이)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북파머스</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>소설</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2024-08-21</t>
+          <t>2024-09-19</t>
         </is>
       </c>
       <c r="G85" t="n">
@@ -4110,29 +4114,25 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>9791193937198</t>
+          <t>9791193937242</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=344497704</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=346467345</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>호감의 시작 (트윙클 에디션)</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>관계, 일, 인생이 풀리는 매력의 법칙</t>
-        </is>
-      </c>
+          <t>빛이 이끄는 곳으로</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
-          <t>희렌최 (지은이)</t>
+          <t>백희성 (지은이)</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4142,47 +4142,47 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>소설</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2024-07-23</t>
+          <t>2024-08-21</t>
         </is>
       </c>
       <c r="G86" t="n">
-        <v>18500</v>
+        <v>18800</v>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>9791193937143</t>
+          <t>9791193937198</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=342932323</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=344497704</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>나는 도대체 왜 피곤할까</t>
+          <t>호감의 시작 (트윙클 에디션)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>이 죽일 놈의 피로와 결별하는 법</t>
+          <t>관계, 일, 인생이 풀리는 매력의 법칙</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>에이미 샤 (지은이), 김잔디 (옮긴이)</t>
+          <t>희렌최 (지은이)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4192,33 +4192,37 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2024-07-10</t>
+          <t>2024-07-23</t>
         </is>
       </c>
       <c r="G87" t="n">
-        <v>19800</v>
+        <v>18500</v>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>9791193937136</t>
+          <t>9791193937143</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=342083093</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=342932323</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>그럼에도 불구하고 나는 내가 좋았어</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
+          <t>나는 도대체 왜 피곤할까</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>이 죽일 놈의 피로와 결별하는 법</t>
+        </is>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>박채린 (지은이)</t>
+          <t>에이미 샤 (지은이), 김잔디 (옮긴이)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4228,102 +4232,98 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2024-06-12</t>
+          <t>2024-07-10</t>
         </is>
       </c>
       <c r="G88" t="n">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>9791193937105</t>
+          <t>9791193937136</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=340511549</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=342083093</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>부자의 마지막 가르침 (30만 부 리커버)</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>삶의 자유를 위한 부의 알고리즘</t>
-        </is>
-      </c>
+          <t>그럼에도 불구하고 나는 내가 좋았어</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
-          <t>다우치 마나부 (지은이), 김슬기 (옮긴이)</t>
+          <t>박채린 (지은이)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2024-05-22</t>
+          <t>2024-06-12</t>
         </is>
       </c>
       <c r="G89" t="n">
-        <v>19800</v>
+        <v>18000</v>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>9791193937068</t>
+          <t>9791193937105</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=363272157</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=340511549</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>똑똑한 아이는 어떻게 생각하고 질문하는가</t>
+          <t>부자의 마지막 가르침 (30만 부 리커버)</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>사고력 실종의 시대, 주도적인 아이들의 생존 전략</t>
+          <t>삶의 자유를 위한 부의 알고리즘</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>이시한 (지은이)</t>
+          <t>다우치 마나부 (지은이), 김슬기 (옮긴이)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>북크레용</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>자녀교육</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2024-05-16</t>
+          <t>2024-05-22</t>
         </is>
       </c>
       <c r="G90" t="n">
@@ -4331,89 +4331,89 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>9791193937037</t>
+          <t>9791193937068</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=337128010</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=363272157</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>사랑받는 이기주의자</t>
+          <t>똑똑한 아이는 어떻게 생각하고 질문하는가</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>나를 지키며 사랑받는 관계의 기술</t>
+          <t>사고력 실종의 시대, 주도적인 아이들의 생존 전략</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>박코 (지은이)</t>
+          <t>이시한 (지은이)</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북크레용</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>자녀교육</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2024-05-02</t>
+          <t>2024-05-16</t>
         </is>
       </c>
       <c r="G91" t="n">
-        <v>18000</v>
+        <v>19800</v>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>9791193937051</t>
+          <t>9791193937037</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=338458067</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=337128010</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>내가 천 개의 인생에서 배운 것들</t>
+          <t>사랑받는 이기주의자</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>돈, 명예, 시간 그 무엇보다 소중한 것에 관하여</t>
+          <t>나를 지키며 사랑받는 관계의 기술</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>김도윤 (지은이)</t>
+          <t>박코 (지은이)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2024-04-17</t>
+          <t>2024-05-02</t>
         </is>
       </c>
       <c r="G92" t="n">
@@ -4421,79 +4421,79 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>9791198530394</t>
+          <t>9791193937051</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=337269711</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=338458067</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>양수인간</t>
+          <t>내가 천 개의 인생에서 배운 것들</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>삶의 격을 높이는 내면 변화 심리학</t>
+          <t>돈, 명예, 시간 그 무엇보다 소중한 것에 관하여</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>최설민 (지은이)</t>
+          <t>김도윤 (지은이)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2024-03-27</t>
+          <t>2024-04-17</t>
         </is>
       </c>
       <c r="G93" t="n">
-        <v>19800</v>
+        <v>18000</v>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>9791193937006</t>
+          <t>9791198530394</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=336173615</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=337269711</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>무엇이 나를 행복하게 만드는가</t>
+          <t>양수인간</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>인생의 절반쯤 왔을 때 깨닫게 되는 것들</t>
+          <t>삶의 격을 높이는 내면 변화 심리학</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>리처드 J. 라이더, 데이비드 A. 샤피로 (지은이), 김정홍 (옮긴이)</t>
+          <t>최설민 (지은이)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>북플레저</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4503,7 +4503,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2024-03-04</t>
+          <t>2024-03-27</t>
         </is>
       </c>
       <c r="G94" t="n">
@@ -4511,29 +4511,29 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>9791198530356</t>
+          <t>9791193937006</t>
         </is>
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=334885758</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=336173615</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>노인의 꿈 : 첫 번째 이야기</t>
+          <t>무엇이 나를 행복하게 만드는가</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>황혼을 향해 걷는 우리 모두의 이야기</t>
+          <t>인생의 절반쯤 왔을 때 깨닫게 되는 것들</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>백원달 (지은이)</t>
+          <t>리처드 J. 라이더, 데이비드 A. 샤피로 (지은이), 김정홍 (옮긴이)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4543,32 +4543,32 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>그 밖의 책</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2024-02-28</t>
+          <t>2024-03-04</t>
         </is>
       </c>
       <c r="G95" t="n">
-        <v>23000</v>
+        <v>19800</v>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>9791191891478</t>
+          <t>9791198530356</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=335184922</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=334885758</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>노인의 꿈 : 두 번째 이야기</t>
+          <t>노인의 꿈 : 첫 번째 이야기</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4601,29 +4601,29 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>9791191891485</t>
+          <t>9791191891478</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=335185323</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=335184922</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>똑똑한 사람은 어떻게 생각하고 질문하는가</t>
+          <t>노인의 꿈 : 두 번째 이야기</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>사고력 실종의 시대, 앞서가는 사람들의 생존 전략</t>
+          <t>황혼을 향해 걷는 우리 모두의 이야기</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>이시한 (지은이)</t>
+          <t>백원달 (지은이)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4633,42 +4633,42 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>그 밖의 책</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2024-01-24</t>
+          <t>2024-02-28</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>19800</v>
+        <v>23000</v>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>9791191891492</t>
+          <t>9791191891485</t>
         </is>
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=332269449</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=335185323</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>산책하듯 가볍게 (풀빛 에디션)</t>
+          <t>똑똑한 사람은 어떻게 생각하고 질문하는가</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>인생에서 여유를 찾는 당신에게 건네는 말</t>
+          <t>사고력 실종의 시대, 앞서가는 사람들의 생존 전략</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>정우성 (지은이)</t>
+          <t>이시한 (지은이)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4678,47 +4678,47 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2023-12-13</t>
+          <t>2024-01-24</t>
         </is>
       </c>
       <c r="G98" t="n">
-        <v>17500</v>
+        <v>19800</v>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>9791191891447</t>
+          <t>9791191891492</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=388109982</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=332269449</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>하는 일마다 잘되리라</t>
+          <t>산책하듯 가볍게 (풀빛 에디션)</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>당신이 어디에 있든 무엇을 하든</t>
+          <t>인생에서 여유를 찾는 당신에게 건네는 말</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>전승환 (지은이)</t>
+          <t>정우성 (지은이)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북플레저</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -4728,127 +4728,127 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2023-11-29</t>
+          <t>2023-12-13</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>18000</v>
+        <v>17500</v>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>9791198530301</t>
+          <t>9791191891447</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=328632910</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=388109982</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>머니 트렌드 2024</t>
+          <t>하는 일마다 잘되리라</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>57가지 키워드로 전망하는 대한민국 돈의 흐름</t>
+          <t>당신이 어디에 있든 무엇을 하든</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>김도윤, 정태익, 김용섭, 김현준, 전영수, 채상욱, 최재붕, 홍춘욱 (지은이)</t>
+          <t>전승환 (지은이)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2023-10-05</t>
+          <t>2023-11-29</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>25000</v>
+        <v>18000</v>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>9791191891416</t>
+          <t>9791198530301</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=324498127</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=328632910</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>꽃은 누구에게나 핀다</t>
+          <t>머니 트렌드 2024</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>오늘부터 내 삶을 바꾸는 자기 확신 에세이, 매일 더 설레는 날을 살게 될 당신에</t>
+          <t>57가지 키워드로 전망하는 대한민국 돈의 흐름</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>오은환 (지은이)</t>
+          <t>김도윤, 정태익, 김용섭, 김현준, 전영수, 채상욱, 최재붕, 홍춘욱 (지은이)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2023-09-19</t>
+          <t>2023-10-05</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>17500</v>
+        <v>25000</v>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>9791191891409</t>
+          <t>9791191891416</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=324723810</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=324498127</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>나는 너랑 노는 게 제일 좋아</t>
+          <t>꽃은 누구에게나 핀다</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>아끼고 고맙고 사랑하는 당신에게</t>
+          <t>오늘부터 내 삶을 바꾸는 자기 확신 에세이, 매일 더 설레는 날을 살게 될 당신에</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>하태완 (지은이)</t>
+          <t>오은환 (지은이)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4863,7 +4863,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2023-07-17</t>
+          <t>2023-09-19</t>
         </is>
       </c>
       <c r="G102" t="n">
@@ -4871,29 +4871,29 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>9791191891362</t>
+          <t>9791191891409</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=320503944</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=324723810</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>마음의 자유</t>
+          <t>나는 너랑 노는 게 제일 좋아</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>행복이란 마음이 어디에도 얽매이지 않는 것</t>
+          <t>아끼고 고맙고 사랑하는 당신에게</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>정윤 (지은이)</t>
+          <t>하태완 (지은이)</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -4908,37 +4908,37 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2023-06-12</t>
+          <t>2023-07-17</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>17000</v>
+        <v>17500</v>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>9791191891355</t>
+          <t>9791191891362</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=318438169</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=320503944</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>찌그러져도 괜찮아</t>
+          <t>마음의 자유</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>이미 찌그러진 오리가</t>
+          <t>행복이란 마음이 어디에도 얽매이지 않는 것</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>찌오(임임) (지은이)</t>
+          <t>정윤 (지은이)</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -4953,7 +4953,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2023-05-02</t>
+          <t>2023-06-12</t>
         </is>
       </c>
       <c r="G104" t="n">
@@ -4961,35 +4961,39 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>9791191891324</t>
+          <t>9791191891355</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=315987317</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=318438169</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>인생에서 가장 후회되는 게 뭐냐고 묻는다면</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr"/>
+          <t>찌그러져도 괜찮아</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>이미 찌그러진 오리가</t>
+        </is>
+      </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>노우티 (지은이)</t>
+          <t>찌오(임임) (지은이)</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>인문·교양</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4998,156 +5002,156 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>17500</v>
+        <v>17000</v>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>9791191891331</t>
+          <t>9791191891324</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=315418702</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=315987317</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>당신과 아침에 싸우면 밤에는 입맞출 겁니다</t>
+          <t>인생에서 가장 후회되는 게 뭐냐고 묻는다면</t>
         </is>
       </c>
       <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
-          <t>유래혁 (지은이)</t>
+          <t>노우티 (지은이)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>인문·교양</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2023-03-20</t>
+          <t>2023-05-02</t>
         </is>
       </c>
       <c r="G106" t="n">
-        <v>17000</v>
+        <v>17500</v>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>9791191891263</t>
+          <t>9791191891331</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=313695065</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=315418702</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GPT 제너레이션 : 챗GPT가 바꿀 우리 인류의 미래</t>
+          <t>당신과 아침에 싸우면 밤에는 입맞출 겁니다</t>
         </is>
       </c>
       <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr">
         <is>
-          <t>이시한 (지은이)</t>
+          <t>유래혁 (지은이)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2023-02-28</t>
+          <t>2023-03-20</t>
         </is>
       </c>
       <c r="G107" t="n">
-        <v>19000</v>
+        <v>17000</v>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>9791191891270</t>
+          <t>9791191891263</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=310813322</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=313695065</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>오둥이입니다만!</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>나는 세상에서 가장 행복한 오리</t>
-        </is>
-      </c>
+          <t>GPT 제너레이션 : 챗GPT가 바꿀 우리 인류의 미래</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
-          <t>송 스튜디오 (지은이)</t>
+          <t>이시한 (지은이)</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2023-02-10</t>
+          <t>2023-02-28</t>
         </is>
       </c>
       <c r="G108" t="n">
-        <v>17000</v>
+        <v>19000</v>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>9791191891256</t>
+          <t>9791191891270</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=310407734</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=310813322</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>행복을 담아줄게</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr"/>
+          <t>오둥이입니다만!</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>나는 세상에서 가장 행복한 오리</t>
+        </is>
+      </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>나란 (지은이)</t>
+          <t>송 스튜디오 (지은이)</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5162,37 +5166,33 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2023-01-30</t>
+          <t>2023-02-10</t>
         </is>
       </c>
       <c r="G109" t="n">
-        <v>16000</v>
+        <v>17000</v>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>9791191891249</t>
+          <t>9791191891256</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=309568882</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=310407734</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>나는 오늘의 내가 좋아</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>긍정토끼 몰랑이의 몰랑몰랑 마음 일기</t>
-        </is>
-      </c>
+          <t>행복을 담아줄게</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
-          <t>윤혜지(하얀오리) (지은이)</t>
+          <t>나란 (지은이)</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2022-12-12</t>
+          <t>2023-01-30</t>
         </is>
       </c>
       <c r="G110" t="n">
@@ -5215,111 +5215,115 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>9791191891126</t>
+          <t>9791191891249</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=306216745</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=309568882</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>머니 트렌드 2023</t>
+          <t>나는 오늘의 내가 좋아</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>45가지 키워드로 전망하는 대한민국 돈의 흐름</t>
+          <t>긍정토끼 몰랑이의 몰랑몰랑 마음 일기</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>부동산읽어주는남자(정태익), 김도윤, 김경민, 김상균, 전영수, 최준철, 홍춘욱 (지은이)</t>
+          <t>윤혜지(하얀오리) (지은이)</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>북모먼트</t>
+          <t>북로망스</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>경제·경영</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2022-11-15</t>
+          <t>2022-12-12</t>
         </is>
       </c>
       <c r="G111" t="n">
-        <v>19000</v>
+        <v>16000</v>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>9791191891232</t>
+          <t>9791191891126</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=304588805</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=306216745</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>잘될 수밖에 없는 너에게</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr"/>
+          <t>머니 트렌드 2023</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>45가지 키워드로 전망하는 대한민국 돈의 흐름</t>
+        </is>
+      </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>최서영 (지은이)</t>
+          <t>부동산읽어주는남자(정태익), 김도윤, 김경민, 김상균, 전영수, 최준철, 홍춘욱 (지은이)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>북로망스</t>
+          <t>북모먼트</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>경제·경영</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2022-08-18</t>
+          <t>2022-11-15</t>
         </is>
       </c>
       <c r="G112" t="n">
-        <v>19500</v>
+        <v>19000</v>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>9791191891201</t>
+          <t>9791191891232</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=299808248</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=304588805</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>나로서 충분히 괜찮은 사람</t>
+          <t>잘될 수밖에 없는 너에게</t>
         </is>
       </c>
       <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
-          <t>김재식 (지은이)</t>
+          <t>최서영 (지은이)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -5334,37 +5338,33 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2022-05-10</t>
+          <t>2022-08-18</t>
         </is>
       </c>
       <c r="G113" t="n">
-        <v>16000</v>
+        <v>19500</v>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>9791191891096</t>
+          <t>9791191891201</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=294392417</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=299808248</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>나에게 고맙다</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>30만 부 기념 전면개정판</t>
-        </is>
-      </c>
+          <t>나로서 충분히 괜찮은 사람</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
-          <t>전승환 (지은이)</t>
+          <t>김재식 (지은이)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -5379,37 +5379,37 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2022-02-18</t>
+          <t>2022-05-10</t>
         </is>
       </c>
       <c r="G114" t="n">
-        <v>19000</v>
+        <v>16000</v>
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>9791191891072</t>
+          <t>9791191891096</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=289269041</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=294392417</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>럭키 LUCKY</t>
+          <t>나에게 고맙다</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>내 안에 잠든 운을 깨우는 7가지 법칙</t>
+          <t>30만 부 기념 전면개정판</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>김도윤 (지은이)</t>
+          <t>전승환 (지은이)</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -5419,42 +5419,42 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>자기계발</t>
+          <t>에세이</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2021-08-25</t>
+          <t>2022-02-18</t>
         </is>
       </c>
       <c r="G115" t="n">
-        <v>20000</v>
+        <v>19000</v>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>9791191891027</t>
+          <t>9791191891072</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=278177114</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=289269041</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>그렇다면 나를 응원할 수밖에 (윈터 에디션)</t>
+          <t>럭키 LUCKY</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>멋대로지만 제대로 사는 중입니다</t>
+          <t>내 안에 잠든 운을 깨우는 7가지 법칙</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>김수민 (지은이)</t>
+          <t>김도윤 (지은이)</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -5464,38 +5464,42 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>에세이</t>
+          <t>자기계발</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2021-07-14</t>
+          <t>2021-08-25</t>
         </is>
       </c>
       <c r="G116" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>9791197037191</t>
+          <t>9791191891027</t>
         </is>
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=283440909</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=278177114</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>작은 별이지만 빛나고 있어 (30만부 기념 미드나잇 에디션)</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr"/>
+          <t>그렇다면 나를 응원할 수밖에 (윈터 에디션)</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>멋대로지만 제대로 사는 중입니다</t>
+        </is>
+      </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>소윤 (지은이)</t>
+          <t>김수민 (지은이)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -5510,33 +5514,33 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2021-03-24</t>
+          <t>2021-07-14</t>
         </is>
       </c>
       <c r="G117" t="n">
-        <v>19000</v>
+        <v>15000</v>
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>9791197037153</t>
+          <t>9791197037191</t>
         </is>
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=367659804</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=283440909</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>좋은 건 같이 봐요</t>
+          <t>작은 별이지만 빛나고 있어 (30만부 기념 미드나잇 에디션)</t>
         </is>
       </c>
       <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
-          <t>엄지사진관 (지은이)</t>
+          <t>소윤 (지은이)</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -5551,33 +5555,33 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2021-01-27</t>
+          <t>2021-03-24</t>
         </is>
       </c>
       <c r="G118" t="n">
-        <v>15000</v>
+        <v>19000</v>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>9791197037146</t>
+          <t>9791197037153</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=262375795</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=367659804</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>안녕, 소중한 사람</t>
+          <t>좋은 건 같이 봐요</t>
         </is>
       </c>
       <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
-          <t>정한경 (지은이)</t>
+          <t>엄지사진관 (지은이)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -5592,63 +5596,104 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2020-09-16</t>
+          <t>2021-01-27</t>
         </is>
       </c>
       <c r="G119" t="n">
-        <v>19000</v>
+        <v>15000</v>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>9791197037122</t>
+          <t>9791197037146</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=251524184</t>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=262375795</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
+          <t>안녕, 소중한 사람</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>정한경 (지은이)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>북로망스</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>에세이</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2020-09-16</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>19000</v>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>9791197037122</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=251524184</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>나는 나를 사랑한다</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>나를 잃지 않고 타인을 사랑하기 위하여</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>이숙명 (지은이)</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>북로망스</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E121" t="inlineStr">
         <is>
           <t>에세이</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F121" t="inlineStr">
         <is>
           <t>2020-06-24</t>
         </is>
       </c>
-      <c r="G120" t="n">
+      <c r="G121" t="n">
         <v>14800</v>
       </c>
-      <c r="H120" t="inlineStr">
+      <c r="H121" t="inlineStr">
         <is>
           <t>9791197037108</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>https://www.aladin.co.kr/shop/wproduct.aspx?ItemId=242494208</t>
         </is>

</xml_diff>

<commit_message>
자동 갱신 2026-10-29 05:20
</commit_message>
<xml_diff>
--- a/files/thebookman-booklist.xlsx
+++ b/files/thebookman-booklist.xlsx
@@ -5811,8 +5811,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Smart, Soulful, and Wholly Me</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>How to live fully as yourself in a world with no right answers.</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>나답게 똘똘하게</t>

</xml_diff>